<commit_message>
Finalizado o catalogo de bicicletas
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael Castro\Documents\catalogo_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06CD26BE-8DF7-4808-93F5-7420EE1B91BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B06F4C8-CB0D-41B9-94BB-908785170714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{02E3CDAF-A272-443C-8687-B38AE8A4CCA2}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="77">
   <si>
     <t>Descrição</t>
   </si>
@@ -51,9 +51,6 @@
     <t>BIC 26 AL VIKING DIRT J.TUFF X-25 AZUL ESCURO/ AMARELO</t>
   </si>
   <si>
-    <t>BICICLETA 26</t>
-  </si>
-  <si>
     <t>83.0446</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>83.0872</t>
   </si>
   <si>
-    <t>BICICLETA 29</t>
-  </si>
-  <si>
     <t>83.0883</t>
   </si>
   <si>
@@ -247,13 +241,31 @@
   </si>
   <si>
     <t>BICICLETA ARO 29 21V FIRST SMITT TAM 19 PRETO F/TIFFANY</t>
+  </si>
+  <si>
+    <t>83.0943</t>
+  </si>
+  <si>
+    <t>BICICLETA ARO 29 24V K7 FIRST LIFTY TAM 17.5 AZUL GALAXY/BRANCO - 54778</t>
+  </si>
+  <si>
+    <t>83.0944</t>
+  </si>
+  <si>
+    <t>BICICLETA ARO 29 24V K7 FIRST LIFTY TAM 17.5 FOSCO GRAFITE/ PRATA - 46904</t>
+  </si>
+  <si>
+    <t>BICICLETAS 26</t>
+  </si>
+  <si>
+    <t>BICICLETAS 29</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -263,12 +275,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -319,13 +325,13 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -640,7 +646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B5E345-C4B2-49FA-A914-04EE787905E0}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -671,566 +677,460 @@
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
       <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
       <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E5" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
       <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E6" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
       <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E7" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
       <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E8" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
       <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E9" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
       <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E10" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
       <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E11" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
       <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E12" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B13" t="s">
-        <v>29</v>
-      </c>
       <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B14" t="s">
-        <v>31</v>
-      </c>
       <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E14" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
       <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E15" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B16" t="s">
-        <v>35</v>
-      </c>
       <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E16" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B17" t="s">
-        <v>37</v>
-      </c>
       <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E17" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="s">
-        <v>39</v>
-      </c>
       <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1145.5</v>
-      </c>
-      <c r="E18" s="2">
-        <v>1064.26</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E19" s="2">
-        <v>692.67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" t="s">
-        <v>45</v>
-      </c>
       <c r="C20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E20" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" t="s">
-        <v>47</v>
+        <v>39</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E21" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" t="s">
-        <v>49</v>
+        <v>44</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E22" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B23" t="s">
-        <v>51</v>
+        <v>46</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E23" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" t="s">
-        <v>53</v>
+        <v>48</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E24" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" t="s">
-        <v>55</v>
+        <v>50</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="C25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E25" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B26" t="s">
-        <v>60</v>
+        <v>52</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
-      </c>
-      <c r="D26" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E26" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" t="s">
-        <v>62</v>
+        <v>57</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E27" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
-      </c>
-      <c r="D28" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E28" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B29" t="s">
-        <v>66</v>
+        <v>61</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="C29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E29" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E30" s="2">
-        <v>692.67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="C31" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E31" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>70</v>
+        <v>54</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>41</v>
-      </c>
-      <c r="D32" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E32" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>71</v>
+        <v>55</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="C33" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E33" s="2">
-        <v>692.67</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C34" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="2">
-        <v>733.64</v>
-      </c>
-      <c r="E34" s="2">
-        <v>692.67</v>
-      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{32B5E345-C4B2-49FA-A914-04EE787905E0}"/>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Criado catalogo de bicicletas com divisorias de especificação
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael Castro\Documents\catalogo_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D75DC4A-3826-4E22-803B-1E6B3C1289C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F13E6B7-CB2B-4453-A3D6-11E87E52FAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{02E3CDAF-A272-443C-8687-B38AE8A4CCA2}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{02E3CDAF-A272-443C-8687-B38AE8A4CCA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="102">
   <si>
     <t>Descrição</t>
   </si>
@@ -322,13 +322,25 @@
   </si>
   <si>
     <t>19 24V</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO BICICLETA 26 VIKING</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO BICICLETA 29 FIRST 21V</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO BICICLETA 29 FIRST 24V</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -341,6 +353,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -389,10 +407,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B5E345-C4B2-49FA-A914-04EE787905E0}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -716,7 +737,7 @@
     <col min="6" max="6" width="21.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -729,8 +750,11 @@
       <c r="F1" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -740,8 +764,11 @@
       <c r="C2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -751,8 +778,11 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -762,8 +792,11 @@
       <c r="C4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -773,8 +806,11 @@
       <c r="C5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -784,8 +820,11 @@
       <c r="C6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -795,8 +834,11 @@
       <c r="C7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -806,8 +848,11 @@
       <c r="C8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -817,8 +862,11 @@
       <c r="C9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -831,8 +879,11 @@
       <c r="F10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>50</v>
       </c>
@@ -845,8 +896,11 @@
       <c r="F11" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -859,8 +913,11 @@
       <c r="F12" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -873,8 +930,11 @@
       <c r="F13" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>39</v>
       </c>
@@ -887,8 +947,11 @@
       <c r="F14" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
@@ -901,8 +964,11 @@
       <c r="F15" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>77</v>
       </c>
@@ -915,8 +981,11 @@
       <c r="F16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -929,8 +998,11 @@
       <c r="F17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>52</v>
       </c>
@@ -943,8 +1015,11 @@
       <c r="F18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>53</v>
       </c>
@@ -957,8 +1032,11 @@
       <c r="F19" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -971,8 +1049,11 @@
       <c r="F20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>54</v>
       </c>
@@ -985,8 +1066,11 @@
       <c r="F21" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>79</v>
       </c>
@@ -999,8 +1083,11 @@
       <c r="F22" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1013,8 +1100,11 @@
       <c r="F23" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
@@ -1027,8 +1117,11 @@
       <c r="F24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>81</v>
       </c>
@@ -1041,8 +1134,11 @@
       <c r="F25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>83</v>
       </c>
@@ -1055,8 +1151,11 @@
       <c r="F26" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>29</v>
       </c>
@@ -1069,8 +1168,11 @@
       <c r="F27" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>85</v>
       </c>
@@ -1083,8 +1185,11 @@
       <c r="F28" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>65</v>
       </c>
@@ -1097,8 +1202,11 @@
       <c r="F29" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>87</v>
       </c>
@@ -1111,8 +1219,11 @@
       <c r="F30">
         <v>19</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
@@ -1125,8 +1236,11 @@
       <c r="F31">
         <v>19</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>69</v>
       </c>
@@ -1139,8 +1253,11 @@
       <c r="F32">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>58</v>
       </c>
@@ -1153,8 +1270,11 @@
       <c r="F33">
         <v>19</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>59</v>
       </c>
@@ -1167,8 +1287,11 @@
       <c r="F34">
         <v>19</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>71</v>
       </c>
@@ -1181,8 +1304,11 @@
       <c r="F35">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>89</v>
       </c>
@@ -1195,8 +1321,11 @@
       <c r="F36">
         <v>19</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -1209,8 +1338,11 @@
       <c r="F37">
         <v>19</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>46</v>
       </c>
@@ -1223,8 +1355,11 @@
       <c r="F38">
         <v>19</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>19</v>
       </c>
@@ -1237,8 +1372,11 @@
       <c r="F39">
         <v>19</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>60</v>
       </c>
@@ -1251,8 +1389,11 @@
       <c r="F40">
         <v>19</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>91</v>
       </c>
@@ -1265,8 +1406,11 @@
       <c r="F41">
         <v>21</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>93</v>
       </c>
@@ -1279,8 +1423,11 @@
       <c r="F42">
         <v>21</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>95</v>
       </c>
@@ -1293,8 +1440,11 @@
       <c r="F43" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>27</v>
       </c>
@@ -1307,8 +1457,11 @@
       <c r="F44" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>11</v>
       </c>
@@ -1320,6 +1473,9 @@
       </c>
       <c r="F45" t="s">
         <v>64</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>